<commit_message>
Add guarded profile editor baseline impact workflow
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="Recd26521703a4720"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="R2304b5c2e9354a78"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R0ef5c894f8ea48a1"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="Rda2db011efcd4617"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="Re2459321ac224684"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="Rad61659c565f4844"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra3656a58efc8410a"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="R77218055b27e4810"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc4bf3ef903b547e9"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R5fd072085f094a6c"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="Rea518725c20b4907"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="R3ad4d67de87c4141"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="Rc80750e94ed143e5"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="R0357963323764849"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="3544ae01-ab54-4b03-9450-04148d0e63c3"/>
+        <xdr:cNvPr id="1" name="4b5f01c2-8e28-48d8-8143-5424b4015d9b"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R97175aa6d9f54ec2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6f045d231ca24286"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R26b78721132347c5"/>
+  <x:drawing ns1:id="R297f19de2f584ee8"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rffced0f786dc4baf"/>
+    <x:tablePart ns1:id="R99a5a32194a24006"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R2c420cc194434f05"/>
+    <x:tablePart ns1:id="R2340c13e8dd14d05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rf2ca06ff9cca49d8"/>
+    <x:tablePart ns1:id="R020519f0ed7a4363"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rb025e9d5cd32400a"/>
+    <x:tablePart ns1:id="Rbbc8483def1944ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6120,7 +6120,7 @@
       </x:c>
       <x:c r="B3" s="99" t="str"/>
       <x:c r="C3" s="99" t="str">
-        <x:v>sha256:68155f752a1bcdfaa7efe2721eec0cd65228e333a447afbd9fe4793d1fc50329</x:v>
+        <x:v>sha256:0cad54af271f69d5d4518d88888c79acc207f64b1538bcc7d6b3fefefdcf8bfd</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
Complete profile editor My Menu workflows
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="R77218055b27e4810"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc4bf3ef903b547e9"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R5fd072085f094a6c"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="Rea518725c20b4907"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="R3ad4d67de87c4141"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="Rc80750e94ed143e5"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="R0357963323764849"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="Rc6435873938f4a68"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc2ece388063b444c"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="Rc376cbfddd3a49b2"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="Rf8c305fc7c564a8e"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="Rf28e705ca5e34901"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R2c389ab70f724530"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="R9d4b0327fe434936"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="4b5f01c2-8e28-48d8-8143-5424b4015d9b"/>
+        <xdr:cNvPr id="1" name="a98550f3-ee28-495b-8e1f-edd7e3eb7e27"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6f045d231ca24286"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R004b67ca2e5844ec"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R297f19de2f584ee8"/>
+  <x:drawing ns1:id="Rf27844338bb5419f"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R99a5a32194a24006"/>
+    <x:tablePart ns1:id="R68db433293694ea3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R2340c13e8dd14d05"/>
+    <x:tablePart ns1:id="R7e30b5f4a5014df2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R020519f0ed7a4363"/>
+    <x:tablePart ns1:id="R4ced039f02a54366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rbbc8483def1944ee"/>
+    <x:tablePart ns1:id="R9d812126885e4251"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6120,7 +6120,7 @@
       </x:c>
       <x:c r="B3" s="99" t="str"/>
       <x:c r="C3" s="99" t="str">
-        <x:v>sha256:0cad54af271f69d5d4518d88888c79acc207f64b1538bcc7d6b3fefefdcf8bfd</x:v>
+        <x:v>sha256:5f5822a7acae425dbb4e9b7323e8bcb7c2933e99c8d0f270d1592e4eac4e883e</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
Keep published docs unchanged during integration
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="Rc6435873938f4a68"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc2ece388063b444c"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="Rc376cbfddd3a49b2"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="Rf8c305fc7c564a8e"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="Rf28e705ca5e34901"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="R2c389ab70f724530"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="R9d4b0327fe434936"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="Recd26521703a4720"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="R2304b5c2e9354a78"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R0ef5c894f8ea48a1"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="Rda2db011efcd4617"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="Re2459321ac224684"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="Rad61659c565f4844"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra3656a58efc8410a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="a98550f3-ee28-495b-8e1f-edd7e3eb7e27"/>
+        <xdr:cNvPr id="1" name="3544ae01-ab54-4b03-9450-04148d0e63c3"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R004b67ca2e5844ec"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R97175aa6d9f54ec2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="Rf27844338bb5419f"/>
+  <x:drawing ns1:id="R26b78721132347c5"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R68db433293694ea3"/>
+    <x:tablePart ns1:id="Rffced0f786dc4baf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R7e30b5f4a5014df2"/>
+    <x:tablePart ns1:id="R2c420cc194434f05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R4ced039f02a54366"/>
+    <x:tablePart ns1:id="Rf2ca06ff9cca49d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R9d812126885e4251"/>
+    <x:tablePart ns1:id="Rb025e9d5cd32400a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6120,7 +6120,7 @@
       </x:c>
       <x:c r="B3" s="99" t="str"/>
       <x:c r="C3" s="99" t="str">
-        <x:v>sha256:5f5822a7acae425dbb4e9b7323e8bcb7c2933e99c8d0f270d1592e4eac4e883e</x:v>
+        <x:v>sha256:68155f752a1bcdfaa7efe2721eec0cd65228e333a447afbd9fe4793d1fc50329</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
Add guarded Cx Foundation workspace
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="Recd26521703a4720"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="R2304b5c2e9354a78"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R0ef5c894f8ea48a1"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="Rda2db011efcd4617"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="Re2459321ac224684"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="Rad61659c565f4844"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra3656a58efc8410a"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="Rc6435873938f4a68"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc2ece388063b444c"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="Rc376cbfddd3a49b2"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="Rf8c305fc7c564a8e"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="Rf28e705ca5e34901"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R2c389ab70f724530"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="R9d4b0327fe434936"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="3544ae01-ab54-4b03-9450-04148d0e63c3"/>
+        <xdr:cNvPr id="1" name="a98550f3-ee28-495b-8e1f-edd7e3eb7e27"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R97175aa6d9f54ec2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R004b67ca2e5844ec"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R26b78721132347c5"/>
+  <x:drawing ns1:id="Rf27844338bb5419f"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rffced0f786dc4baf"/>
+    <x:tablePart ns1:id="R68db433293694ea3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R2c420cc194434f05"/>
+    <x:tablePart ns1:id="R7e30b5f4a5014df2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rf2ca06ff9cca49d8"/>
+    <x:tablePart ns1:id="R4ced039f02a54366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rb025e9d5cd32400a"/>
+    <x:tablePart ns1:id="R9d812126885e4251"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6120,7 +6120,7 @@
       </x:c>
       <x:c r="B3" s="99" t="str"/>
       <x:c r="C3" s="99" t="str">
-        <x:v>sha256:68155f752a1bcdfaa7efe2721eec0cd65228e333a447afbd9fe4793d1fc50329</x:v>
+        <x:v>sha256:5f5822a7acae425dbb4e9b7323e8bcb7c2933e99c8d0f270d1592e4eac4e883e</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
Align Cx routes and validation artifacts
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="Rc6435873938f4a68"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc2ece388063b444c"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="Rc376cbfddd3a49b2"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="Rf8c305fc7c564a8e"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="Rf28e705ca5e34901"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="R2c389ab70f724530"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="R9d4b0327fe434936"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="R3b4624d52a354fff"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="R17c924773ef144b0"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R47b2830b56fd4eab"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="R50e330cbaa7e4f24"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="R380a0179589e4f13"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R0f34f017b6dc4fc6"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra5a9ab3bf42d4f71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="a98550f3-ee28-495b-8e1f-edd7e3eb7e27"/>
+        <xdr:cNvPr id="1" name="62a24901-1ef3-4ff1-adba-3a249c35557d"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R004b67ca2e5844ec"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d94f8ca10b6403d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="Rf27844338bb5419f"/>
+  <x:drawing ns1:id="Rdf37c0e7b43b47e1"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R68db433293694ea3"/>
+    <x:tablePart ns1:id="Re5b60396c6d745a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R7e30b5f4a5014df2"/>
+    <x:tablePart ns1:id="R9ec7d47d58de443d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R4ced039f02a54366"/>
+    <x:tablePart ns1:id="R6e27681e97e548e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R9d812126885e4251"/>
+    <x:tablePart ns1:id="Rd14a0597aa0048b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Integrate Profile Editor with Camera Lab
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="R3b4624d52a354fff"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="R17c924773ef144b0"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R47b2830b56fd4eab"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="R50e330cbaa7e4f24"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="R380a0179589e4f13"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="R0f34f017b6dc4fc6"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra5a9ab3bf42d4f71"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="Rc6435873938f4a68"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc2ece388063b444c"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="Rc376cbfddd3a49b2"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="Rf8c305fc7c564a8e"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="Rf28e705ca5e34901"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R2c389ab70f724530"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="R9d4b0327fe434936"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="62a24901-1ef3-4ff1-adba-3a249c35557d"/>
+        <xdr:cNvPr id="1" name="a98550f3-ee28-495b-8e1f-edd7e3eb7e27"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d94f8ca10b6403d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R004b67ca2e5844ec"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="Rdf37c0e7b43b47e1"/>
+  <x:drawing ns1:id="Rf27844338bb5419f"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Re5b60396c6d745a4"/>
+    <x:tablePart ns1:id="R68db433293694ea3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R9ec7d47d58de443d"/>
+    <x:tablePart ns1:id="R7e30b5f4a5014df2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R6e27681e97e548e8"/>
+    <x:tablePart ns1:id="R4ced039f02a54366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rd14a0597aa0048b8"/>
+    <x:tablePart ns1:id="R9d812126885e4251"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh main verification downloads
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="Rc6435873938f4a68"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="Rc2ece388063b444c"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="Rc376cbfddd3a49b2"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="Rf8c305fc7c564a8e"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="Rf28e705ca5e34901"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="R2c389ab70f724530"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="R9d4b0327fe434936"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="R3b4624d52a354fff"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="R17c924773ef144b0"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R47b2830b56fd4eab"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="R50e330cbaa7e4f24"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="R380a0179589e4f13"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R0f34f017b6dc4fc6"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra5a9ab3bf42d4f71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="a98550f3-ee28-495b-8e1f-edd7e3eb7e27"/>
+        <xdr:cNvPr id="1" name="62a24901-1ef3-4ff1-adba-3a249c35557d"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R004b67ca2e5844ec"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d94f8ca10b6403d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="Rf27844338bb5419f"/>
+  <x:drawing ns1:id="Rdf37c0e7b43b47e1"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R68db433293694ea3"/>
+    <x:tablePart ns1:id="Re5b60396c6d745a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R7e30b5f4a5014df2"/>
+    <x:tablePart ns1:id="R9ec7d47d58de443d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R4ced039f02a54366"/>
+    <x:tablePart ns1:id="R6e27681e97e548e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R9d812126885e4251"/>
+    <x:tablePart ns1:id="Rd14a0597aa0048b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Finalize profile catalog and isolate pack roots
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="R3b4624d52a354fff"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="R17c924773ef144b0"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R47b2830b56fd4eab"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="R50e330cbaa7e4f24"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="R380a0179589e4f13"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="R0f34f017b6dc4fc6"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra5a9ab3bf42d4f71"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="R652895637daa487c"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="R594c446137cc4cac"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R0260dc22b23d40d1"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="R3a8aae84195f42a3"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="R865ac3c4c3a8485c"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R934677c968d640cd"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="R9e32fb1623594543"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="62a24901-1ef3-4ff1-adba-3a249c35557d"/>
+        <xdr:cNvPr id="1" name="547f717f-9c71-4eab-8f9c-a606ce33b96e"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d94f8ca10b6403d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6665a6309014528"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="Rdf37c0e7b43b47e1"/>
+  <x:drawing ns1:id="R4ba3a0213cea4066"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Re5b60396c6d745a4"/>
+    <x:tablePart ns1:id="Rf00f98d73cdb4ecd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R9ec7d47d58de443d"/>
+    <x:tablePart ns1:id="Rce19ceaabda14f84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R6e27681e97e548e8"/>
+    <x:tablePart ns1:id="R9fafa41c0b3c42ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rd14a0597aa0048b8"/>
+    <x:tablePart ns1:id="R958a2fe5e2764966"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6111,27 +6111,25 @@
       </x:c>
       <x:c r="B2" s="99" t="str"/>
       <x:c r="C2" s="99" t="str">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="99" t="str">
-        <x:v>source_fingerprint</x:v>
+        <x:v>spreadsheet_build_id</x:v>
       </x:c>
       <x:c r="B3" s="99" t="str"/>
       <x:c r="C3" s="99" t="str">
-        <x:v>sha256:5f5822a7acae425dbb4e9b7323e8bcb7c2933e99c8d0f270d1592e4eac4e883e</x:v>
+        <x:v>S3-08d641519318</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="99" t="str">
-        <x:v>test</x:v>
-      </x:c>
-      <x:c r="B4" s="99" t="str">
-        <x:v>SETUP-01</x:v>
-      </x:c>
+        <x:v>source_fingerprint</x:v>
+      </x:c>
+      <x:c r="B4" s="99" t="str"/>
       <x:c r="C4" s="99" t="str">
-        <x:v>sha256:6298d64e10367b2e38e5d41253bb816c1012479ab7612afc5a53ad66630e975f</x:v>
+        <x:v>sha256:08d6415193181337fead9371040d20422e94b4ed704294692294a69805dca6db</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6139,10 +6137,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B5" s="99" t="str">
-        <x:v>SETUP-02</x:v>
+        <x:v>SETUP-01</x:v>
       </x:c>
       <x:c r="C5" s="99" t="str">
-        <x:v>sha256:2c28c37a65e2efee3349ec9d9c3a6e75de10e76697f1c3b5ec5ca8d1ceae0030</x:v>
+        <x:v>sha256:6298d64e10367b2e38e5d41253bb816c1012479ab7612afc5a53ad66630e975f</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6150,10 +6148,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B6" s="99" t="str">
-        <x:v>SETUP-03</x:v>
+        <x:v>SETUP-02</x:v>
       </x:c>
       <x:c r="C6" s="99" t="str">
-        <x:v>sha256:eb596d6e2a1ad3dba500a053b487e07af4813566f59012575380f500c95740a3</x:v>
+        <x:v>sha256:2c28c37a65e2efee3349ec9d9c3a6e75de10e76697f1c3b5ec5ca8d1ceae0030</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -6161,10 +6159,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B7" s="99" t="str">
-        <x:v>SETUP-MM-01</x:v>
+        <x:v>SETUP-03</x:v>
       </x:c>
       <x:c r="C7" s="99" t="str">
-        <x:v>sha256:c760cc1bea9609da89be5d36089ba2323849d51903b5f40f43c986536aab0cc0</x:v>
+        <x:v>sha256:eb596d6e2a1ad3dba500a053b487e07af4813566f59012575380f500c95740a3</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6172,10 +6170,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B8" s="99" t="str">
-        <x:v>SETUP-MM-AF-01</x:v>
+        <x:v>SETUP-MM-01</x:v>
       </x:c>
       <x:c r="C8" s="99" t="str">
-        <x:v>sha256:2b88f49e05b245e31f0d823f6ef4e5d71a2bd0398b2cf9cd8205610832364ab9</x:v>
+        <x:v>sha256:c760cc1bea9609da89be5d36089ba2323849d51903b5f40f43c986536aab0cc0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6183,10 +6181,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B9" s="99" t="str">
-        <x:v>SETUP-04</x:v>
+        <x:v>SETUP-MM-AF-01</x:v>
       </x:c>
       <x:c r="C9" s="99" t="str">
-        <x:v>sha256:b6bd467f6a89f821e9373cc530c60d121981c3be1f93118148955e75331daaa4</x:v>
+        <x:v>sha256:2b88f49e05b245e31f0d823f6ef4e5d71a2bd0398b2cf9cd8205610832364ab9</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6194,10 +6192,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B10" s="99" t="str">
-        <x:v>SETUP-05</x:v>
+        <x:v>SETUP-04</x:v>
       </x:c>
       <x:c r="C10" s="99" t="str">
-        <x:v>sha256:67ea99e7324822765d73c9e1a978991ba090dd1fcb01bc4f819eb693e2018f1b</x:v>
+        <x:v>sha256:b6bd467f6a89f821e9373cc530c60d121981c3be1f93118148955e75331daaa4</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6205,10 +6203,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B11" s="99" t="str">
-        <x:v>SETUP-06</x:v>
+        <x:v>SETUP-05</x:v>
       </x:c>
       <x:c r="C11" s="99" t="str">
-        <x:v>sha256:50a7bb1d684b76be2ecaf5dd70540adcc5036481c265a2d6e4348a13c0d3f061</x:v>
+        <x:v>sha256:67ea99e7324822765d73c9e1a978991ba090dd1fcb01bc4f819eb693e2018f1b</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6216,10 +6214,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B12" s="99" t="str">
-        <x:v>SETUP-07</x:v>
+        <x:v>SETUP-06</x:v>
       </x:c>
       <x:c r="C12" s="99" t="str">
-        <x:v>sha256:4465ab573d202c4fbb497291b08a1c5ffffad91c48872e300991471bef2567f4</x:v>
+        <x:v>sha256:50a7bb1d684b76be2ecaf5dd70540adcc5036481c265a2d6e4348a13c0d3f061</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6227,10 +6225,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B13" s="99" t="str">
-        <x:v>CTRL-CONFIG-01</x:v>
+        <x:v>SETUP-07</x:v>
       </x:c>
       <x:c r="C13" s="99" t="str">
-        <x:v>sha256:bf207e6d54b48768207e423d534c48709f88f234d55bdcb9613e260a68c411f2</x:v>
+        <x:v>sha256:4465ab573d202c4fbb497291b08a1c5ffffad91c48872e300991471bef2567f4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -6238,10 +6236,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B14" s="99" t="str">
-        <x:v>BACKUP-SET-01</x:v>
+        <x:v>CTRL-CONFIG-01</x:v>
       </x:c>
       <x:c r="C14" s="99" t="str">
-        <x:v>sha256:a17b1005496620e34a1ee11e646e9a1fc082c4eb20ac617592011ba5e6ceae8a</x:v>
+        <x:v>sha256:bf207e6d54b48768207e423d534c48709f88f234d55bdcb9613e260a68c411f2</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6249,10 +6247,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B15" s="99" t="str">
-        <x:v>C1-CONFIG-01</x:v>
+        <x:v>BACKUP-SET-01</x:v>
       </x:c>
       <x:c r="C15" s="99" t="str">
-        <x:v>sha256:1507d79e9f067c7c5b2099b8101a3d17938d127abce04324c2c3ac3d6b72efd7</x:v>
+        <x:v>sha256:a17b1005496620e34a1ee11e646e9a1fc082c4eb20ac617592011ba5e6ceae8a</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6260,10 +6258,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B16" s="99" t="str">
-        <x:v>C1-REG-01</x:v>
+        <x:v>C1-CONFIG-01</x:v>
       </x:c>
       <x:c r="C16" s="99" t="str">
-        <x:v>sha256:04a561cd1850599049f01a2ec97355afe25fe8c5fc4c4c81d52f639897d63b03</x:v>
+        <x:v>sha256:1507d79e9f067c7c5b2099b8101a3d17938d127abce04324c2c3ac3d6b72efd7</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6271,10 +6269,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B17" s="99" t="str">
-        <x:v>C1-READ-01</x:v>
+        <x:v>C1-REG-01</x:v>
       </x:c>
       <x:c r="C17" s="99" t="str">
-        <x:v>sha256:2c25a1c907b5edcc56c06bd4e4bd1d8dde41fa6faebde85baec2ab4a2acefd87</x:v>
+        <x:v>sha256:04a561cd1850599049f01a2ec97355afe25fe8c5fc4c4c81d52f639897d63b03</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6282,10 +6280,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B18" s="99" t="str">
-        <x:v>C1-OPS-01</x:v>
+        <x:v>C1-READ-01</x:v>
       </x:c>
       <x:c r="C18" s="99" t="str">
-        <x:v>sha256:88304c030b7adb56fe9666b1d5541eb373d1615173ce399a06f9538b960dfc1e</x:v>
+        <x:v>sha256:2c25a1c907b5edcc56c06bd4e4bd1d8dde41fa6faebde85baec2ab4a2acefd87</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -6293,10 +6291,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B19" s="99" t="str">
-        <x:v>C2-CONFIG-01</x:v>
+        <x:v>C1-OPS-01</x:v>
       </x:c>
       <x:c r="C19" s="99" t="str">
-        <x:v>sha256:cb99fda58735522dedf306188a4a8f12400a51676d686f840b660c38650789c3</x:v>
+        <x:v>sha256:88304c030b7adb56fe9666b1d5541eb373d1615173ce399a06f9538b960dfc1e</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6304,10 +6302,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B20" s="99" t="str">
-        <x:v>C2-REG-01</x:v>
+        <x:v>C2-CONFIG-01</x:v>
       </x:c>
       <x:c r="C20" s="99" t="str">
-        <x:v>sha256:f4b28c92d9a20605b591f5721dd3ad3beff4e7b5105c8c15a65d23398e8e2d56</x:v>
+        <x:v>sha256:cb99fda58735522dedf306188a4a8f12400a51676d686f840b660c38650789c3</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -6315,10 +6313,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B21" s="99" t="str">
-        <x:v>C2-READ-01</x:v>
+        <x:v>C2-REG-01</x:v>
       </x:c>
       <x:c r="C21" s="99" t="str">
-        <x:v>sha256:cda561c58eb3b3eeb7b5d8b86836960a48f9ee79058073e4943561aa9c9b39d1</x:v>
+        <x:v>sha256:f4b28c92d9a20605b591f5721dd3ad3beff4e7b5105c8c15a65d23398e8e2d56</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6326,10 +6324,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B22" s="99" t="str">
-        <x:v>C2-OPS-01</x:v>
+        <x:v>C2-READ-01</x:v>
       </x:c>
       <x:c r="C22" s="99" t="str">
-        <x:v>sha256:d939e6407cadc5480c2f88547845d69f1e2e36a37b7ae6635cebcdde0e9ce030</x:v>
+        <x:v>sha256:cda561c58eb3b3eeb7b5d8b86836960a48f9ee79058073e4943561aa9c9b39d1</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6337,10 +6335,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B23" s="99" t="str">
-        <x:v>C3-CONFIG-01</x:v>
+        <x:v>C2-OPS-01</x:v>
       </x:c>
       <x:c r="C23" s="99" t="str">
-        <x:v>sha256:633063511fb285503511b318ef26bf092ac48be8afda4df5ef008ab645d4f712</x:v>
+        <x:v>sha256:d939e6407cadc5480c2f88547845d69f1e2e36a37b7ae6635cebcdde0e9ce030</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6348,10 +6346,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B24" s="99" t="str">
-        <x:v>C3-REG-01</x:v>
+        <x:v>C3-CONFIG-01</x:v>
       </x:c>
       <x:c r="C24" s="99" t="str">
-        <x:v>sha256:f692886e78e72d84e31a5ef91aa281938d0529b8b7ea1a220bbf200993144e29</x:v>
+        <x:v>sha256:633063511fb285503511b318ef26bf092ac48be8afda4df5ef008ab645d4f712</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6359,10 +6357,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B25" s="99" t="str">
-        <x:v>C3-READ-01</x:v>
+        <x:v>C3-REG-01</x:v>
       </x:c>
       <x:c r="C25" s="99" t="str">
-        <x:v>sha256:44b63514e2b1f8af98d36c6a4a25a22b7d554a7055c63b717a390b5801f4f72f</x:v>
+        <x:v>sha256:f692886e78e72d84e31a5ef91aa281938d0529b8b7ea1a220bbf200993144e29</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -6370,10 +6368,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B26" s="99" t="str">
-        <x:v>BACKUP-SET-02</x:v>
+        <x:v>C3-READ-01</x:v>
       </x:c>
       <x:c r="C26" s="99" t="str">
-        <x:v>sha256:d8e92939499af335b6f4493b97c7fa8671ad4fc3910cca9a5f8eda4ef41cfc2f</x:v>
+        <x:v>sha256:44b63514e2b1f8af98d36c6a4a25a22b7d554a7055c63b717a390b5801f4f72f</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -6381,10 +6379,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B27" s="99" t="str">
-        <x:v>C3-OPS-01</x:v>
+        <x:v>BACKUP-SET-02</x:v>
       </x:c>
       <x:c r="C27" s="99" t="str">
-        <x:v>sha256:c60f649504d508a81fa0bd19f172421676472153728093142a04d2ba4e5c96ad</x:v>
+        <x:v>sha256:d8e92939499af335b6f4493b97c7fa8671ad4fc3910cca9a5f8eda4ef41cfc2f</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -6392,10 +6390,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B28" s="99" t="str">
-        <x:v>CTRL-AFON-01</x:v>
+        <x:v>C3-OPS-01</x:v>
       </x:c>
       <x:c r="C28" s="99" t="str">
-        <x:v>sha256:2c3055256d014c23ff48c71e8998a544186d8606fc4ad766773ec6c14976f6d7</x:v>
+        <x:v>sha256:c60f649504d508a81fa0bd19f172421676472153728093142a04d2ba4e5c96ad</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -6403,10 +6401,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B29" s="99" t="str">
-        <x:v>CTRL-AELOCK-01</x:v>
+        <x:v>CTRL-AFON-01</x:v>
       </x:c>
       <x:c r="C29" s="99" t="str">
-        <x:v>sha256:888daf7bc311ea1a395e8a7406c8caac4655da1853803ba28df50d40a03fda9b</x:v>
+        <x:v>sha256:2c3055256d014c23ff48c71e8998a544186d8606fc4ad766773ec6c14976f6d7</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -6414,10 +6412,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B30" s="99" t="str">
-        <x:v>CTRL-DOF-01</x:v>
+        <x:v>CTRL-AELOCK-01</x:v>
       </x:c>
       <x:c r="C30" s="99" t="str">
-        <x:v>sha256:606ba83c6c6ef93bebe9f6f0451a7c80fead0f83b62fd48fe2137c5a72fa3b19</x:v>
+        <x:v>sha256:888daf7bc311ea1a395e8a7406c8caac4655da1853803ba28df50d40a03fda9b</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -6425,10 +6423,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B31" s="99" t="str">
-        <x:v>CTRL-SET-01</x:v>
+        <x:v>CTRL-DOF-01</x:v>
       </x:c>
       <x:c r="C31" s="99" t="str">
-        <x:v>sha256:ad0d38b06de1f9f53cde8acce71775385e4aaef6588e771934320e4124431e25</x:v>
+        <x:v>sha256:606ba83c6c6ef93bebe9f6f0451a7c80fead0f83b62fd48fe2137c5a72fa3b19</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -6436,10 +6434,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B32" s="99" t="str">
-        <x:v>CTRL-JOY-01</x:v>
+        <x:v>CTRL-SET-01</x:v>
       </x:c>
       <x:c r="C32" s="99" t="str">
-        <x:v>sha256:957387ec73ac18ab4785a4aaf972f7e285c513c90769f009edece0c97f044600</x:v>
+        <x:v>sha256:ad0d38b06de1f9f53cde8acce71775385e4aaef6588e771934320e4124431e25</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -6447,10 +6445,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B33" s="99" t="str">
-        <x:v>EFCS-SHOCK-01</x:v>
+        <x:v>CTRL-JOY-01</x:v>
       </x:c>
       <x:c r="C33" s="99" t="str">
-        <x:v>sha256:5536143e9808461e6a2779baa6f8d2adf0dd969cccb0b7d2a28598a924d61203</x:v>
+        <x:v>sha256:957387ec73ac18ab4785a4aaf972f7e285c513c90769f009edece0c97f044600</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -6458,10 +6456,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B34" s="99" t="str">
-        <x:v>EFCS-BOKEH-01</x:v>
+        <x:v>EFCS-SHOCK-01</x:v>
       </x:c>
       <x:c r="C34" s="99" t="str">
-        <x:v>sha256:4e1bd076174191e3341b0eb9a6f2279f745b35cc3425dbd6e1360e771e5f3a42</x:v>
+        <x:v>sha256:5536143e9808461e6a2779baa6f8d2adf0dd969cccb0b7d2a28598a924d61203</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -6469,10 +6467,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B35" s="99" t="str">
-        <x:v>EFCS-LIGHT-01</x:v>
+        <x:v>EFCS-BOKEH-01</x:v>
       </x:c>
       <x:c r="C35" s="99" t="str">
-        <x:v>sha256:0294347c51bd94b65f8eec9fad44b39d00e5433c4dc12aeee06c48c0e5ae9c08</x:v>
+        <x:v>sha256:4e1bd076174191e3341b0eb9a6f2279f745b35cc3425dbd6e1360e771e5f3a42</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -6480,10 +6478,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B36" s="99" t="str">
-        <x:v>EFCS-BURST-01</x:v>
+        <x:v>EFCS-LIGHT-01</x:v>
       </x:c>
       <x:c r="C36" s="99" t="str">
-        <x:v>sha256:10966e281790e9619773bd99c263d1a8c3f83170403b36c2fbb2a490499e7130</x:v>
+        <x:v>sha256:0294347c51bd94b65f8eec9fad44b39d00e5433c4dc12aeee06c48c0e5ae9c08</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -6491,10 +6489,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B37" s="99" t="str">
-        <x:v>FLASH-PLUTO-01</x:v>
+        <x:v>EFCS-BURST-01</x:v>
       </x:c>
       <x:c r="C37" s="99" t="str">
-        <x:v>sha256:5c00b09991f26e6b8bedd930e7304b53dae8f93819c7135c765aac82e970d87c</x:v>
+        <x:v>sha256:10966e281790e9619773bd99c263d1a8c3f83170403b36c2fbb2a490499e7130</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -6502,10 +6500,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B38" s="99" t="str">
-        <x:v>FINAL-READ-01</x:v>
+        <x:v>FLASH-PLUTO-01</x:v>
       </x:c>
       <x:c r="C38" s="99" t="str">
-        <x:v>sha256:688b6db6bd3d38070dfd682da54402cf8678093cb1014766953f9f5da49d7407</x:v>
+        <x:v>sha256:5c00b09991f26e6b8bedd930e7304b53dae8f93819c7135c765aac82e970d87c</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -6513,10 +6511,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B39" s="99" t="str">
-        <x:v>FINAL-SAVE-01</x:v>
+        <x:v>FINAL-READ-01</x:v>
       </x:c>
       <x:c r="C39" s="99" t="str">
-        <x:v>sha256:3d3558eaa54a0fdee859a544db2bccada6d3a8749fda96001422741914b6d0a6</x:v>
+        <x:v>sha256:688b6db6bd3d38070dfd682da54402cf8678093cb1014766953f9f5da49d7407</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -6524,21 +6522,21 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B40" s="99" t="str">
-        <x:v>PROJECT-UPDATE-01</x:v>
+        <x:v>FINAL-SAVE-01</x:v>
       </x:c>
       <x:c r="C40" s="99" t="str">
-        <x:v>sha256:9312ccf684ccf233900950855d7a3457eb01e52e1c8fcb90e3c7c7daa72e17a6</x:v>
+        <x:v>sha256:3d3558eaa54a0fdee859a544db2bccada6d3a8749fda96001422741914b6d0a6</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="99" t="str">
-        <x:v>registration</x:v>
+        <x:v>test</x:v>
       </x:c>
       <x:c r="B41" s="99" t="str">
-        <x:v>Mode</x:v>
+        <x:v>PROJECT-UPDATE-01</x:v>
       </x:c>
       <x:c r="C41" s="99" t="str">
-        <x:v>sha256:16380d447ae550758ff49c344119374224a6b1c009504e23f6f4f93c11c00533</x:v>
+        <x:v>sha256:9312ccf684ccf233900950855d7a3457eb01e52e1c8fcb90e3c7c7daa72e17a6</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -6546,10 +6544,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B42" s="99" t="str">
-        <x:v>Metering</x:v>
+        <x:v>Mode</x:v>
       </x:c>
       <x:c r="C42" s="99" t="str">
-        <x:v>sha256:bc76af3dd5f76e718fe876deafcfbc0fd4a3f64d2a2eb64d2253751bd18f4eae</x:v>
+        <x:v>sha256:16380d447ae550758ff49c344119374224a6b1c009504e23f6f4f93c11c00533</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -6557,10 +6555,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B43" s="99" t="str">
-        <x:v>Exposure Compensation</x:v>
+        <x:v>Metering</x:v>
       </x:c>
       <x:c r="C43" s="99" t="str">
-        <x:v>sha256:88e1331bb1792dc8c402253666af51d91b4ff14bdf848d8f5715f7c5735374ee</x:v>
+        <x:v>sha256:bc76af3dd5f76e718fe876deafcfbc0fd4a3f64d2a2eb64d2253751bd18f4eae</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -6568,10 +6566,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B44" s="99" t="str">
-        <x:v>Shutter Speed</x:v>
+        <x:v>Exposure Compensation</x:v>
       </x:c>
       <x:c r="C44" s="99" t="str">
-        <x:v>sha256:50a59b23cd80339f63a7068a9f9b6618357bcc05eb6f986cc5c7a707e50c0a74</x:v>
+        <x:v>sha256:88e1331bb1792dc8c402253666af51d91b4ff14bdf848d8f5715f7c5735374ee</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -6579,10 +6577,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B45" s="99" t="str">
-        <x:v>Aperture</x:v>
+        <x:v>Shutter Speed</x:v>
       </x:c>
       <x:c r="C45" s="99" t="str">
-        <x:v>sha256:74b8c602aefe9109b324a5d3d0f5af54cafeaceae6f80e96effd7b7e7b7512a0</x:v>
+        <x:v>sha256:50a59b23cd80339f63a7068a9f9b6618357bcc05eb6f986cc5c7a707e50c0a74</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -6590,10 +6588,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B46" s="99" t="str">
-        <x:v>ISO</x:v>
+        <x:v>Aperture</x:v>
       </x:c>
       <x:c r="C46" s="99" t="str">
-        <x:v>sha256:3c57560fdad255af8dddd4afe759bf3a638ced62cd0b435fbcb39f539ed4d5cd</x:v>
+        <x:v>sha256:74b8c602aefe9109b324a5d3d0f5af54cafeaceae6f80e96effd7b7e7b7512a0</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -6601,10 +6599,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B47" s="99" t="str">
-        <x:v>Auto ISO Maximum</x:v>
+        <x:v>ISO</x:v>
       </x:c>
       <x:c r="C47" s="99" t="str">
-        <x:v>sha256:215087f96f2c5d379e4931bbcffe7ea4f1ebe59cc0229f5dae23f52e08edbba5</x:v>
+        <x:v>sha256:3c57560fdad255af8dddd4afe759bf3a638ced62cd0b435fbcb39f539ed4d5cd</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -6612,10 +6610,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B48" s="99" t="str">
-        <x:v>AF Operation</x:v>
+        <x:v>Auto ISO Maximum</x:v>
       </x:c>
       <x:c r="C48" s="99" t="str">
-        <x:v>sha256:e52a8877636b9e990324e5e59a10b6b8a0723c7699f752ac41a4e39a25ed8c94</x:v>
+        <x:v>sha256:215087f96f2c5d379e4931bbcffe7ea4f1ebe59cc0229f5dae23f52e08edbba5</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -6623,10 +6621,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B49" s="99" t="str">
-        <x:v>Servo AF Case</x:v>
+        <x:v>AF Operation</x:v>
       </x:c>
       <x:c r="C49" s="99" t="str">
-        <x:v>sha256:c9f1ca7567fd410ce854474a770e020fea6e9904b6872801ebc1b2f20b392fbf</x:v>
+        <x:v>sha256:e52a8877636b9e990324e5e59a10b6b8a0723c7699f752ac41a4e39a25ed8c94</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -6634,10 +6632,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B50" s="99" t="str">
-        <x:v>Tracking Sensitivity</x:v>
+        <x:v>Servo AF Case</x:v>
       </x:c>
       <x:c r="C50" s="99" t="str">
-        <x:v>sha256:dfe83819227cc879db8a3ff1c5b898a2d1c1b0f74d6b3364ad9a92ed7b018424</x:v>
+        <x:v>sha256:c9f1ca7567fd410ce854474a770e020fea6e9904b6872801ebc1b2f20b392fbf</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -6645,10 +6643,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B51" s="99" t="str">
-        <x:v>Accel./Decel. Tracking</x:v>
+        <x:v>Tracking Sensitivity</x:v>
       </x:c>
       <x:c r="C51" s="99" t="str">
-        <x:v>sha256:e11fda77b702b46abfbda7bbf4de92c162668fd479106b46da999dcd11ba28cf</x:v>
+        <x:v>sha256:dfe83819227cc879db8a3ff1c5b898a2d1c1b0f74d6b3364ad9a92ed7b018424</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -6656,10 +6654,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B52" s="99" t="str">
-        <x:v>Switching Tracked Subjects</x:v>
+        <x:v>Accel./Decel. Tracking</x:v>
       </x:c>
       <x:c r="C52" s="99" t="str">
-        <x:v>sha256:1866e2e49cd4159a2f76e301df8394efb14ebc00f49606d84fedb5501875eeb7</x:v>
+        <x:v>sha256:e11fda77b702b46abfbda7bbf4de92c162668fd479106b46da999dcd11ba28cf</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -6667,10 +6665,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B53" s="99" t="str">
-        <x:v>AF Method</x:v>
+        <x:v>Switching Tracked Subjects</x:v>
       </x:c>
       <x:c r="C53" s="99" t="str">
-        <x:v>sha256:ac30ce5e48a2e9e69db02806afb6a8c836dd8220dce399b57ed50b6ec3569d82</x:v>
+        <x:v>sha256:1866e2e49cd4159a2f76e301df8394efb14ebc00f49606d84fedb5501875eeb7</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -6678,10 +6676,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B54" s="99" t="str">
-        <x:v>Subject Detection</x:v>
+        <x:v>AF Method</x:v>
       </x:c>
       <x:c r="C54" s="99" t="str">
-        <x:v>sha256:ca630f9c8761b1ba9bc261fc0264e1fdff6c6ebce7d3d60f68453c6e6c0fb66e</x:v>
+        <x:v>sha256:ac30ce5e48a2e9e69db02806afb6a8c836dd8220dce399b57ed50b6ec3569d82</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -6689,10 +6687,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B55" s="99" t="str">
-        <x:v>Eye Detection</x:v>
+        <x:v>Subject Detection</x:v>
       </x:c>
       <x:c r="C55" s="99" t="str">
-        <x:v>sha256:d4f49e58f189bc2a85058e8030bdba5867549892594d4961911a877fc7774cc1</x:v>
+        <x:v>sha256:ca630f9c8761b1ba9bc261fc0264e1fdff6c6ebce7d3d60f68453c6e6c0fb66e</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -6700,10 +6698,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B56" s="99" t="str">
-        <x:v>Drive Mode</x:v>
+        <x:v>Eye Detection</x:v>
       </x:c>
       <x:c r="C56" s="99" t="str">
-        <x:v>sha256:a407ab25d86c6b32e4618dffadce1bc9f7375731cceb32a9b15154cb636bbc93</x:v>
+        <x:v>sha256:d4f49e58f189bc2a85058e8030bdba5867549892594d4961911a877fc7774cc1</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -6711,10 +6709,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B57" s="99" t="str">
-        <x:v>High Speed Display</x:v>
+        <x:v>Drive Mode</x:v>
       </x:c>
       <x:c r="C57" s="99" t="str">
-        <x:v>sha256:0af962b70870008b8b495ab863d5b9773e68daa4e052c10a5157bbb6e9b09a04</x:v>
+        <x:v>sha256:a407ab25d86c6b32e4618dffadce1bc9f7375731cceb32a9b15154cb636bbc93</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -6722,10 +6720,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B58" s="99" t="str">
-        <x:v>Shutter Type</x:v>
+        <x:v>High Speed Display</x:v>
       </x:c>
       <x:c r="C58" s="99" t="str">
-        <x:v>sha256:e0eb3a601149113b744968c8d35c10e22707716e94c780644837edcabff082bb</x:v>
+        <x:v>sha256:0af962b70870008b8b495ab863d5b9773e68daa4e052c10a5157bbb6e9b09a04</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -6733,10 +6731,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B59" s="99" t="str">
-        <x:v>Image Stabilizer Mode</x:v>
+        <x:v>Shutter Type</x:v>
       </x:c>
       <x:c r="C59" s="99" t="str">
-        <x:v>sha256:cc5907ea77c17b747bda000cb9d24e886022b15d9be9b15be2fd7d3a6aa18fba</x:v>
+        <x:v>sha256:e0eb3a601149113b744968c8d35c10e22707716e94c780644837edcabff082bb</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -6744,10 +6742,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B60" s="99" t="str">
-        <x:v>IBIS</x:v>
+        <x:v>Image Stabilizer Mode</x:v>
       </x:c>
       <x:c r="C60" s="99" t="str">
-        <x:v>sha256:f88432494f6ce6fd467acf866dcb7285209af0daa97f23211b4c2e9a2fca510a</x:v>
+        <x:v>sha256:cc5907ea77c17b747bda000cb9d24e886022b15d9be9b15be2fd7d3a6aa18fba</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -6755,10 +6753,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B61" s="99" t="str">
-        <x:v>Focus Bracketing</x:v>
+        <x:v>IBIS</x:v>
       </x:c>
       <x:c r="C61" s="99" t="str">
-        <x:v>sha256:faa653558ccc3ca42def02cffceb2449676221f3e2b701a95cb76c734a606a66</x:v>
+        <x:v>sha256:f88432494f6ce6fd467acf866dcb7285209af0daa97f23211b4c2e9a2fca510a</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -6766,9 +6764,20 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B62" s="99" t="str">
+        <x:v>Focus Bracketing</x:v>
+      </x:c>
+      <x:c r="C62" s="99" t="str">
+        <x:v>sha256:faa653558ccc3ca42def02cffceb2449676221f3e2b701a95cb76c734a606a66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="99" t="str">
+        <x:v>registration</x:v>
+      </x:c>
+      <x:c r="B63" s="99" t="str">
         <x:v>Lens IS switch</x:v>
       </x:c>
-      <x:c r="C62" s="99" t="str">
+      <x:c r="C63" s="99" t="str">
         <x:v>sha256:77c1f08d541f8a95c354155213e1184f193765664d2faca4e6245806067b6735</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Remove generated website changes from integration
</commit_message>
<xml_diff>
--- a/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
+++ b/docs/downloads/EOS R5 Setup & Verification Tracker.xlsx
@@ -5,13 +5,13 @@
     <x:workbookView activeTab="0"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Dashboard" sheetId="1" ns1:id="R652895637daa487c"/>
-    <x:sheet name="Checklist" sheetId="2" ns1:id="R594c446137cc4cac"/>
-    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R0260dc22b23d40d1"/>
-    <x:sheet name="Sessions" sheetId="4" ns1:id="R3a8aae84195f42a3"/>
-    <x:sheet name="Lists" sheetId="5" ns1:id="R865ac3c4c3a8485c"/>
-    <x:sheet name="Menu" sheetId="6" ns1:id="R934677c968d640cd"/>
-    <x:sheet name="Metadata" sheetId="7" ns1:id="R9e32fb1623594543"/>
+    <x:sheet name="Dashboard" sheetId="1" ns1:id="R3b4624d52a354fff"/>
+    <x:sheet name="Checklist" sheetId="2" ns1:id="R17c924773ef144b0"/>
+    <x:sheet name="C1-C3 Registration" sheetId="3" ns1:id="R47b2830b56fd4eab"/>
+    <x:sheet name="Sessions" sheetId="4" ns1:id="R50e330cbaa7e4f24"/>
+    <x:sheet name="Lists" sheetId="5" ns1:id="R380a0179589e4f13"/>
+    <x:sheet name="Menu" sheetId="6" ns1:id="R0f34f017b6dc4fc6"/>
+    <x:sheet name="Metadata" sheetId="7" ns1:id="Ra5a9ab3bf42d4f71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,13 +704,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="547f717f-9c71-4eab-8f9c-a606ce33b96e"/>
+        <xdr:cNvPr id="1" name="62a24901-1ef3-4ff1-adba-3a249c35557d"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6665a6309014528"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d94f8ca10b6403d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3486,9 +3486,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R4ba3a0213cea4066"/>
+  <x:drawing ns1:id="Rdf37c0e7b43b47e1"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rf00f98d73cdb4ecd"/>
+    <x:tablePart ns1:id="Re5b60396c6d745a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4877,7 +4877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rce19ceaabda14f84"/>
+    <x:tablePart ns1:id="R9ec7d47d58de443d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5258,7 +5258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R9fafa41c0b3c42ff"/>
+    <x:tablePart ns1:id="R6e27681e97e548e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6080,7 +6080,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R958a2fe5e2764966"/>
+    <x:tablePart ns1:id="Rd14a0597aa0048b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6111,25 +6111,27 @@
       </x:c>
       <x:c r="B2" s="99" t="str"/>
       <x:c r="C2" s="99" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="99" t="str">
-        <x:v>spreadsheet_build_id</x:v>
+        <x:v>source_fingerprint</x:v>
       </x:c>
       <x:c r="B3" s="99" t="str"/>
       <x:c r="C3" s="99" t="str">
-        <x:v>S3-08d641519318</x:v>
+        <x:v>sha256:5f5822a7acae425dbb4e9b7323e8bcb7c2933e99c8d0f270d1592e4eac4e883e</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="99" t="str">
-        <x:v>source_fingerprint</x:v>
-      </x:c>
-      <x:c r="B4" s="99" t="str"/>
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="B4" s="99" t="str">
+        <x:v>SETUP-01</x:v>
+      </x:c>
       <x:c r="C4" s="99" t="str">
-        <x:v>sha256:08d6415193181337fead9371040d20422e94b4ed704294692294a69805dca6db</x:v>
+        <x:v>sha256:6298d64e10367b2e38e5d41253bb816c1012479ab7612afc5a53ad66630e975f</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6137,10 +6139,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B5" s="99" t="str">
-        <x:v>SETUP-01</x:v>
+        <x:v>SETUP-02</x:v>
       </x:c>
       <x:c r="C5" s="99" t="str">
-        <x:v>sha256:6298d64e10367b2e38e5d41253bb816c1012479ab7612afc5a53ad66630e975f</x:v>
+        <x:v>sha256:2c28c37a65e2efee3349ec9d9c3a6e75de10e76697f1c3b5ec5ca8d1ceae0030</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6148,10 +6150,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B6" s="99" t="str">
-        <x:v>SETUP-02</x:v>
+        <x:v>SETUP-03</x:v>
       </x:c>
       <x:c r="C6" s="99" t="str">
-        <x:v>sha256:2c28c37a65e2efee3349ec9d9c3a6e75de10e76697f1c3b5ec5ca8d1ceae0030</x:v>
+        <x:v>sha256:eb596d6e2a1ad3dba500a053b487e07af4813566f59012575380f500c95740a3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -6159,10 +6161,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B7" s="99" t="str">
-        <x:v>SETUP-03</x:v>
+        <x:v>SETUP-MM-01</x:v>
       </x:c>
       <x:c r="C7" s="99" t="str">
-        <x:v>sha256:eb596d6e2a1ad3dba500a053b487e07af4813566f59012575380f500c95740a3</x:v>
+        <x:v>sha256:c760cc1bea9609da89be5d36089ba2323849d51903b5f40f43c986536aab0cc0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6170,10 +6172,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B8" s="99" t="str">
-        <x:v>SETUP-MM-01</x:v>
+        <x:v>SETUP-MM-AF-01</x:v>
       </x:c>
       <x:c r="C8" s="99" t="str">
-        <x:v>sha256:c760cc1bea9609da89be5d36089ba2323849d51903b5f40f43c986536aab0cc0</x:v>
+        <x:v>sha256:2b88f49e05b245e31f0d823f6ef4e5d71a2bd0398b2cf9cd8205610832364ab9</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6181,10 +6183,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B9" s="99" t="str">
-        <x:v>SETUP-MM-AF-01</x:v>
+        <x:v>SETUP-04</x:v>
       </x:c>
       <x:c r="C9" s="99" t="str">
-        <x:v>sha256:2b88f49e05b245e31f0d823f6ef4e5d71a2bd0398b2cf9cd8205610832364ab9</x:v>
+        <x:v>sha256:b6bd467f6a89f821e9373cc530c60d121981c3be1f93118148955e75331daaa4</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6192,10 +6194,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B10" s="99" t="str">
-        <x:v>SETUP-04</x:v>
+        <x:v>SETUP-05</x:v>
       </x:c>
       <x:c r="C10" s="99" t="str">
-        <x:v>sha256:b6bd467f6a89f821e9373cc530c60d121981c3be1f93118148955e75331daaa4</x:v>
+        <x:v>sha256:67ea99e7324822765d73c9e1a978991ba090dd1fcb01bc4f819eb693e2018f1b</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6203,10 +6205,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B11" s="99" t="str">
-        <x:v>SETUP-05</x:v>
+        <x:v>SETUP-06</x:v>
       </x:c>
       <x:c r="C11" s="99" t="str">
-        <x:v>sha256:67ea99e7324822765d73c9e1a978991ba090dd1fcb01bc4f819eb693e2018f1b</x:v>
+        <x:v>sha256:50a7bb1d684b76be2ecaf5dd70540adcc5036481c265a2d6e4348a13c0d3f061</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6214,10 +6216,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B12" s="99" t="str">
-        <x:v>SETUP-06</x:v>
+        <x:v>SETUP-07</x:v>
       </x:c>
       <x:c r="C12" s="99" t="str">
-        <x:v>sha256:50a7bb1d684b76be2ecaf5dd70540adcc5036481c265a2d6e4348a13c0d3f061</x:v>
+        <x:v>sha256:4465ab573d202c4fbb497291b08a1c5ffffad91c48872e300991471bef2567f4</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6225,10 +6227,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B13" s="99" t="str">
-        <x:v>SETUP-07</x:v>
+        <x:v>CTRL-CONFIG-01</x:v>
       </x:c>
       <x:c r="C13" s="99" t="str">
-        <x:v>sha256:4465ab573d202c4fbb497291b08a1c5ffffad91c48872e300991471bef2567f4</x:v>
+        <x:v>sha256:bf207e6d54b48768207e423d534c48709f88f234d55bdcb9613e260a68c411f2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -6236,10 +6238,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B14" s="99" t="str">
-        <x:v>CTRL-CONFIG-01</x:v>
+        <x:v>BACKUP-SET-01</x:v>
       </x:c>
       <x:c r="C14" s="99" t="str">
-        <x:v>sha256:bf207e6d54b48768207e423d534c48709f88f234d55bdcb9613e260a68c411f2</x:v>
+        <x:v>sha256:a17b1005496620e34a1ee11e646e9a1fc082c4eb20ac617592011ba5e6ceae8a</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6247,10 +6249,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B15" s="99" t="str">
-        <x:v>BACKUP-SET-01</x:v>
+        <x:v>C1-CONFIG-01</x:v>
       </x:c>
       <x:c r="C15" s="99" t="str">
-        <x:v>sha256:a17b1005496620e34a1ee11e646e9a1fc082c4eb20ac617592011ba5e6ceae8a</x:v>
+        <x:v>sha256:1507d79e9f067c7c5b2099b8101a3d17938d127abce04324c2c3ac3d6b72efd7</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6258,10 +6260,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B16" s="99" t="str">
-        <x:v>C1-CONFIG-01</x:v>
+        <x:v>C1-REG-01</x:v>
       </x:c>
       <x:c r="C16" s="99" t="str">
-        <x:v>sha256:1507d79e9f067c7c5b2099b8101a3d17938d127abce04324c2c3ac3d6b72efd7</x:v>
+        <x:v>sha256:04a561cd1850599049f01a2ec97355afe25fe8c5fc4c4c81d52f639897d63b03</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6269,10 +6271,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B17" s="99" t="str">
-        <x:v>C1-REG-01</x:v>
+        <x:v>C1-READ-01</x:v>
       </x:c>
       <x:c r="C17" s="99" t="str">
-        <x:v>sha256:04a561cd1850599049f01a2ec97355afe25fe8c5fc4c4c81d52f639897d63b03</x:v>
+        <x:v>sha256:2c25a1c907b5edcc56c06bd4e4bd1d8dde41fa6faebde85baec2ab4a2acefd87</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6280,10 +6282,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B18" s="99" t="str">
-        <x:v>C1-READ-01</x:v>
+        <x:v>C1-OPS-01</x:v>
       </x:c>
       <x:c r="C18" s="99" t="str">
-        <x:v>sha256:2c25a1c907b5edcc56c06bd4e4bd1d8dde41fa6faebde85baec2ab4a2acefd87</x:v>
+        <x:v>sha256:88304c030b7adb56fe9666b1d5541eb373d1615173ce399a06f9538b960dfc1e</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -6291,10 +6293,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B19" s="99" t="str">
-        <x:v>C1-OPS-01</x:v>
+        <x:v>C2-CONFIG-01</x:v>
       </x:c>
       <x:c r="C19" s="99" t="str">
-        <x:v>sha256:88304c030b7adb56fe9666b1d5541eb373d1615173ce399a06f9538b960dfc1e</x:v>
+        <x:v>sha256:cb99fda58735522dedf306188a4a8f12400a51676d686f840b660c38650789c3</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6302,10 +6304,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B20" s="99" t="str">
-        <x:v>C2-CONFIG-01</x:v>
+        <x:v>C2-REG-01</x:v>
       </x:c>
       <x:c r="C20" s="99" t="str">
-        <x:v>sha256:cb99fda58735522dedf306188a4a8f12400a51676d686f840b660c38650789c3</x:v>
+        <x:v>sha256:f4b28c92d9a20605b591f5721dd3ad3beff4e7b5105c8c15a65d23398e8e2d56</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -6313,10 +6315,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B21" s="99" t="str">
-        <x:v>C2-REG-01</x:v>
+        <x:v>C2-READ-01</x:v>
       </x:c>
       <x:c r="C21" s="99" t="str">
-        <x:v>sha256:f4b28c92d9a20605b591f5721dd3ad3beff4e7b5105c8c15a65d23398e8e2d56</x:v>
+        <x:v>sha256:cda561c58eb3b3eeb7b5d8b86836960a48f9ee79058073e4943561aa9c9b39d1</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6324,10 +6326,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B22" s="99" t="str">
-        <x:v>C2-READ-01</x:v>
+        <x:v>C2-OPS-01</x:v>
       </x:c>
       <x:c r="C22" s="99" t="str">
-        <x:v>sha256:cda561c58eb3b3eeb7b5d8b86836960a48f9ee79058073e4943561aa9c9b39d1</x:v>
+        <x:v>sha256:d939e6407cadc5480c2f88547845d69f1e2e36a37b7ae6635cebcdde0e9ce030</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6335,10 +6337,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B23" s="99" t="str">
-        <x:v>C2-OPS-01</x:v>
+        <x:v>C3-CONFIG-01</x:v>
       </x:c>
       <x:c r="C23" s="99" t="str">
-        <x:v>sha256:d939e6407cadc5480c2f88547845d69f1e2e36a37b7ae6635cebcdde0e9ce030</x:v>
+        <x:v>sha256:633063511fb285503511b318ef26bf092ac48be8afda4df5ef008ab645d4f712</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6346,10 +6348,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B24" s="99" t="str">
-        <x:v>C3-CONFIG-01</x:v>
+        <x:v>C3-REG-01</x:v>
       </x:c>
       <x:c r="C24" s="99" t="str">
-        <x:v>sha256:633063511fb285503511b318ef26bf092ac48be8afda4df5ef008ab645d4f712</x:v>
+        <x:v>sha256:f692886e78e72d84e31a5ef91aa281938d0529b8b7ea1a220bbf200993144e29</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6357,10 +6359,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B25" s="99" t="str">
-        <x:v>C3-REG-01</x:v>
+        <x:v>C3-READ-01</x:v>
       </x:c>
       <x:c r="C25" s="99" t="str">
-        <x:v>sha256:f692886e78e72d84e31a5ef91aa281938d0529b8b7ea1a220bbf200993144e29</x:v>
+        <x:v>sha256:44b63514e2b1f8af98d36c6a4a25a22b7d554a7055c63b717a390b5801f4f72f</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -6368,10 +6370,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B26" s="99" t="str">
-        <x:v>C3-READ-01</x:v>
+        <x:v>BACKUP-SET-02</x:v>
       </x:c>
       <x:c r="C26" s="99" t="str">
-        <x:v>sha256:44b63514e2b1f8af98d36c6a4a25a22b7d554a7055c63b717a390b5801f4f72f</x:v>
+        <x:v>sha256:d8e92939499af335b6f4493b97c7fa8671ad4fc3910cca9a5f8eda4ef41cfc2f</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -6379,10 +6381,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B27" s="99" t="str">
-        <x:v>BACKUP-SET-02</x:v>
+        <x:v>C3-OPS-01</x:v>
       </x:c>
       <x:c r="C27" s="99" t="str">
-        <x:v>sha256:d8e92939499af335b6f4493b97c7fa8671ad4fc3910cca9a5f8eda4ef41cfc2f</x:v>
+        <x:v>sha256:c60f649504d508a81fa0bd19f172421676472153728093142a04d2ba4e5c96ad</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -6390,10 +6392,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B28" s="99" t="str">
-        <x:v>C3-OPS-01</x:v>
+        <x:v>CTRL-AFON-01</x:v>
       </x:c>
       <x:c r="C28" s="99" t="str">
-        <x:v>sha256:c60f649504d508a81fa0bd19f172421676472153728093142a04d2ba4e5c96ad</x:v>
+        <x:v>sha256:2c3055256d014c23ff48c71e8998a544186d8606fc4ad766773ec6c14976f6d7</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -6401,10 +6403,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B29" s="99" t="str">
-        <x:v>CTRL-AFON-01</x:v>
+        <x:v>CTRL-AELOCK-01</x:v>
       </x:c>
       <x:c r="C29" s="99" t="str">
-        <x:v>sha256:2c3055256d014c23ff48c71e8998a544186d8606fc4ad766773ec6c14976f6d7</x:v>
+        <x:v>sha256:888daf7bc311ea1a395e8a7406c8caac4655da1853803ba28df50d40a03fda9b</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -6412,10 +6414,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B30" s="99" t="str">
-        <x:v>CTRL-AELOCK-01</x:v>
+        <x:v>CTRL-DOF-01</x:v>
       </x:c>
       <x:c r="C30" s="99" t="str">
-        <x:v>sha256:888daf7bc311ea1a395e8a7406c8caac4655da1853803ba28df50d40a03fda9b</x:v>
+        <x:v>sha256:606ba83c6c6ef93bebe9f6f0451a7c80fead0f83b62fd48fe2137c5a72fa3b19</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -6423,10 +6425,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B31" s="99" t="str">
-        <x:v>CTRL-DOF-01</x:v>
+        <x:v>CTRL-SET-01</x:v>
       </x:c>
       <x:c r="C31" s="99" t="str">
-        <x:v>sha256:606ba83c6c6ef93bebe9f6f0451a7c80fead0f83b62fd48fe2137c5a72fa3b19</x:v>
+        <x:v>sha256:ad0d38b06de1f9f53cde8acce71775385e4aaef6588e771934320e4124431e25</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -6434,10 +6436,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B32" s="99" t="str">
-        <x:v>CTRL-SET-01</x:v>
+        <x:v>CTRL-JOY-01</x:v>
       </x:c>
       <x:c r="C32" s="99" t="str">
-        <x:v>sha256:ad0d38b06de1f9f53cde8acce71775385e4aaef6588e771934320e4124431e25</x:v>
+        <x:v>sha256:957387ec73ac18ab4785a4aaf972f7e285c513c90769f009edece0c97f044600</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -6445,10 +6447,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B33" s="99" t="str">
-        <x:v>CTRL-JOY-01</x:v>
+        <x:v>EFCS-SHOCK-01</x:v>
       </x:c>
       <x:c r="C33" s="99" t="str">
-        <x:v>sha256:957387ec73ac18ab4785a4aaf972f7e285c513c90769f009edece0c97f044600</x:v>
+        <x:v>sha256:5536143e9808461e6a2779baa6f8d2adf0dd969cccb0b7d2a28598a924d61203</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -6456,10 +6458,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B34" s="99" t="str">
-        <x:v>EFCS-SHOCK-01</x:v>
+        <x:v>EFCS-BOKEH-01</x:v>
       </x:c>
       <x:c r="C34" s="99" t="str">
-        <x:v>sha256:5536143e9808461e6a2779baa6f8d2adf0dd969cccb0b7d2a28598a924d61203</x:v>
+        <x:v>sha256:4e1bd076174191e3341b0eb9a6f2279f745b35cc3425dbd6e1360e771e5f3a42</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -6467,10 +6469,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B35" s="99" t="str">
-        <x:v>EFCS-BOKEH-01</x:v>
+        <x:v>EFCS-LIGHT-01</x:v>
       </x:c>
       <x:c r="C35" s="99" t="str">
-        <x:v>sha256:4e1bd076174191e3341b0eb9a6f2279f745b35cc3425dbd6e1360e771e5f3a42</x:v>
+        <x:v>sha256:0294347c51bd94b65f8eec9fad44b39d00e5433c4dc12aeee06c48c0e5ae9c08</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -6478,10 +6480,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B36" s="99" t="str">
-        <x:v>EFCS-LIGHT-01</x:v>
+        <x:v>EFCS-BURST-01</x:v>
       </x:c>
       <x:c r="C36" s="99" t="str">
-        <x:v>sha256:0294347c51bd94b65f8eec9fad44b39d00e5433c4dc12aeee06c48c0e5ae9c08</x:v>
+        <x:v>sha256:10966e281790e9619773bd99c263d1a8c3f83170403b36c2fbb2a490499e7130</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -6489,10 +6491,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B37" s="99" t="str">
-        <x:v>EFCS-BURST-01</x:v>
+        <x:v>FLASH-PLUTO-01</x:v>
       </x:c>
       <x:c r="C37" s="99" t="str">
-        <x:v>sha256:10966e281790e9619773bd99c263d1a8c3f83170403b36c2fbb2a490499e7130</x:v>
+        <x:v>sha256:5c00b09991f26e6b8bedd930e7304b53dae8f93819c7135c765aac82e970d87c</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -6500,10 +6502,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B38" s="99" t="str">
-        <x:v>FLASH-PLUTO-01</x:v>
+        <x:v>FINAL-READ-01</x:v>
       </x:c>
       <x:c r="C38" s="99" t="str">
-        <x:v>sha256:5c00b09991f26e6b8bedd930e7304b53dae8f93819c7135c765aac82e970d87c</x:v>
+        <x:v>sha256:688b6db6bd3d38070dfd682da54402cf8678093cb1014766953f9f5da49d7407</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -6511,10 +6513,10 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B39" s="99" t="str">
-        <x:v>FINAL-READ-01</x:v>
+        <x:v>FINAL-SAVE-01</x:v>
       </x:c>
       <x:c r="C39" s="99" t="str">
-        <x:v>sha256:688b6db6bd3d38070dfd682da54402cf8678093cb1014766953f9f5da49d7407</x:v>
+        <x:v>sha256:3d3558eaa54a0fdee859a544db2bccada6d3a8749fda96001422741914b6d0a6</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -6522,21 +6524,21 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="B40" s="99" t="str">
-        <x:v>FINAL-SAVE-01</x:v>
+        <x:v>PROJECT-UPDATE-01</x:v>
       </x:c>
       <x:c r="C40" s="99" t="str">
-        <x:v>sha256:3d3558eaa54a0fdee859a544db2bccada6d3a8749fda96001422741914b6d0a6</x:v>
+        <x:v>sha256:9312ccf684ccf233900950855d7a3457eb01e52e1c8fcb90e3c7c7daa72e17a6</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="99" t="str">
-        <x:v>test</x:v>
+        <x:v>registration</x:v>
       </x:c>
       <x:c r="B41" s="99" t="str">
-        <x:v>PROJECT-UPDATE-01</x:v>
+        <x:v>Mode</x:v>
       </x:c>
       <x:c r="C41" s="99" t="str">
-        <x:v>sha256:9312ccf684ccf233900950855d7a3457eb01e52e1c8fcb90e3c7c7daa72e17a6</x:v>
+        <x:v>sha256:16380d447ae550758ff49c344119374224a6b1c009504e23f6f4f93c11c00533</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -6544,10 +6546,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B42" s="99" t="str">
-        <x:v>Mode</x:v>
+        <x:v>Metering</x:v>
       </x:c>
       <x:c r="C42" s="99" t="str">
-        <x:v>sha256:16380d447ae550758ff49c344119374224a6b1c009504e23f6f4f93c11c00533</x:v>
+        <x:v>sha256:bc76af3dd5f76e718fe876deafcfbc0fd4a3f64d2a2eb64d2253751bd18f4eae</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -6555,10 +6557,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B43" s="99" t="str">
-        <x:v>Metering</x:v>
+        <x:v>Exposure Compensation</x:v>
       </x:c>
       <x:c r="C43" s="99" t="str">
-        <x:v>sha256:bc76af3dd5f76e718fe876deafcfbc0fd4a3f64d2a2eb64d2253751bd18f4eae</x:v>
+        <x:v>sha256:88e1331bb1792dc8c402253666af51d91b4ff14bdf848d8f5715f7c5735374ee</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -6566,10 +6568,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B44" s="99" t="str">
-        <x:v>Exposure Compensation</x:v>
+        <x:v>Shutter Speed</x:v>
       </x:c>
       <x:c r="C44" s="99" t="str">
-        <x:v>sha256:88e1331bb1792dc8c402253666af51d91b4ff14bdf848d8f5715f7c5735374ee</x:v>
+        <x:v>sha256:50a59b23cd80339f63a7068a9f9b6618357bcc05eb6f986cc5c7a707e50c0a74</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -6577,10 +6579,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B45" s="99" t="str">
-        <x:v>Shutter Speed</x:v>
+        <x:v>Aperture</x:v>
       </x:c>
       <x:c r="C45" s="99" t="str">
-        <x:v>sha256:50a59b23cd80339f63a7068a9f9b6618357bcc05eb6f986cc5c7a707e50c0a74</x:v>
+        <x:v>sha256:74b8c602aefe9109b324a5d3d0f5af54cafeaceae6f80e96effd7b7e7b7512a0</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -6588,10 +6590,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B46" s="99" t="str">
-        <x:v>Aperture</x:v>
+        <x:v>ISO</x:v>
       </x:c>
       <x:c r="C46" s="99" t="str">
-        <x:v>sha256:74b8c602aefe9109b324a5d3d0f5af54cafeaceae6f80e96effd7b7e7b7512a0</x:v>
+        <x:v>sha256:3c57560fdad255af8dddd4afe759bf3a638ced62cd0b435fbcb39f539ed4d5cd</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -6599,10 +6601,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B47" s="99" t="str">
-        <x:v>ISO</x:v>
+        <x:v>Auto ISO Maximum</x:v>
       </x:c>
       <x:c r="C47" s="99" t="str">
-        <x:v>sha256:3c57560fdad255af8dddd4afe759bf3a638ced62cd0b435fbcb39f539ed4d5cd</x:v>
+        <x:v>sha256:215087f96f2c5d379e4931bbcffe7ea4f1ebe59cc0229f5dae23f52e08edbba5</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -6610,10 +6612,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B48" s="99" t="str">
-        <x:v>Auto ISO Maximum</x:v>
+        <x:v>AF Operation</x:v>
       </x:c>
       <x:c r="C48" s="99" t="str">
-        <x:v>sha256:215087f96f2c5d379e4931bbcffe7ea4f1ebe59cc0229f5dae23f52e08edbba5</x:v>
+        <x:v>sha256:e52a8877636b9e990324e5e59a10b6b8a0723c7699f752ac41a4e39a25ed8c94</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -6621,10 +6623,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B49" s="99" t="str">
-        <x:v>AF Operation</x:v>
+        <x:v>Servo AF Case</x:v>
       </x:c>
       <x:c r="C49" s="99" t="str">
-        <x:v>sha256:e52a8877636b9e990324e5e59a10b6b8a0723c7699f752ac41a4e39a25ed8c94</x:v>
+        <x:v>sha256:c9f1ca7567fd410ce854474a770e020fea6e9904b6872801ebc1b2f20b392fbf</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -6632,10 +6634,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B50" s="99" t="str">
-        <x:v>Servo AF Case</x:v>
+        <x:v>Tracking Sensitivity</x:v>
       </x:c>
       <x:c r="C50" s="99" t="str">
-        <x:v>sha256:c9f1ca7567fd410ce854474a770e020fea6e9904b6872801ebc1b2f20b392fbf</x:v>
+        <x:v>sha256:dfe83819227cc879db8a3ff1c5b898a2d1c1b0f74d6b3364ad9a92ed7b018424</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -6643,10 +6645,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B51" s="99" t="str">
-        <x:v>Tracking Sensitivity</x:v>
+        <x:v>Accel./Decel. Tracking</x:v>
       </x:c>
       <x:c r="C51" s="99" t="str">
-        <x:v>sha256:dfe83819227cc879db8a3ff1c5b898a2d1c1b0f74d6b3364ad9a92ed7b018424</x:v>
+        <x:v>sha256:e11fda77b702b46abfbda7bbf4de92c162668fd479106b46da999dcd11ba28cf</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -6654,10 +6656,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B52" s="99" t="str">
-        <x:v>Accel./Decel. Tracking</x:v>
+        <x:v>Switching Tracked Subjects</x:v>
       </x:c>
       <x:c r="C52" s="99" t="str">
-        <x:v>sha256:e11fda77b702b46abfbda7bbf4de92c162668fd479106b46da999dcd11ba28cf</x:v>
+        <x:v>sha256:1866e2e49cd4159a2f76e301df8394efb14ebc00f49606d84fedb5501875eeb7</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -6665,10 +6667,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B53" s="99" t="str">
-        <x:v>Switching Tracked Subjects</x:v>
+        <x:v>AF Method</x:v>
       </x:c>
       <x:c r="C53" s="99" t="str">
-        <x:v>sha256:1866e2e49cd4159a2f76e301df8394efb14ebc00f49606d84fedb5501875eeb7</x:v>
+        <x:v>sha256:ac30ce5e48a2e9e69db02806afb6a8c836dd8220dce399b57ed50b6ec3569d82</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -6676,10 +6678,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B54" s="99" t="str">
-        <x:v>AF Method</x:v>
+        <x:v>Subject Detection</x:v>
       </x:c>
       <x:c r="C54" s="99" t="str">
-        <x:v>sha256:ac30ce5e48a2e9e69db02806afb6a8c836dd8220dce399b57ed50b6ec3569d82</x:v>
+        <x:v>sha256:ca630f9c8761b1ba9bc261fc0264e1fdff6c6ebce7d3d60f68453c6e6c0fb66e</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -6687,10 +6689,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B55" s="99" t="str">
-        <x:v>Subject Detection</x:v>
+        <x:v>Eye Detection</x:v>
       </x:c>
       <x:c r="C55" s="99" t="str">
-        <x:v>sha256:ca630f9c8761b1ba9bc261fc0264e1fdff6c6ebce7d3d60f68453c6e6c0fb66e</x:v>
+        <x:v>sha256:d4f49e58f189bc2a85058e8030bdba5867549892594d4961911a877fc7774cc1</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -6698,10 +6700,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B56" s="99" t="str">
-        <x:v>Eye Detection</x:v>
+        <x:v>Drive Mode</x:v>
       </x:c>
       <x:c r="C56" s="99" t="str">
-        <x:v>sha256:d4f49e58f189bc2a85058e8030bdba5867549892594d4961911a877fc7774cc1</x:v>
+        <x:v>sha256:a407ab25d86c6b32e4618dffadce1bc9f7375731cceb32a9b15154cb636bbc93</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -6709,10 +6711,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B57" s="99" t="str">
-        <x:v>Drive Mode</x:v>
+        <x:v>High Speed Display</x:v>
       </x:c>
       <x:c r="C57" s="99" t="str">
-        <x:v>sha256:a407ab25d86c6b32e4618dffadce1bc9f7375731cceb32a9b15154cb636bbc93</x:v>
+        <x:v>sha256:0af962b70870008b8b495ab863d5b9773e68daa4e052c10a5157bbb6e9b09a04</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -6720,10 +6722,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B58" s="99" t="str">
-        <x:v>High Speed Display</x:v>
+        <x:v>Shutter Type</x:v>
       </x:c>
       <x:c r="C58" s="99" t="str">
-        <x:v>sha256:0af962b70870008b8b495ab863d5b9773e68daa4e052c10a5157bbb6e9b09a04</x:v>
+        <x:v>sha256:e0eb3a601149113b744968c8d35c10e22707716e94c780644837edcabff082bb</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -6731,10 +6733,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B59" s="99" t="str">
-        <x:v>Shutter Type</x:v>
+        <x:v>Image Stabilizer Mode</x:v>
       </x:c>
       <x:c r="C59" s="99" t="str">
-        <x:v>sha256:e0eb3a601149113b744968c8d35c10e22707716e94c780644837edcabff082bb</x:v>
+        <x:v>sha256:cc5907ea77c17b747bda000cb9d24e886022b15d9be9b15be2fd7d3a6aa18fba</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -6742,10 +6744,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B60" s="99" t="str">
-        <x:v>Image Stabilizer Mode</x:v>
+        <x:v>IBIS</x:v>
       </x:c>
       <x:c r="C60" s="99" t="str">
-        <x:v>sha256:cc5907ea77c17b747bda000cb9d24e886022b15d9be9b15be2fd7d3a6aa18fba</x:v>
+        <x:v>sha256:f88432494f6ce6fd467acf866dcb7285209af0daa97f23211b4c2e9a2fca510a</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -6753,10 +6755,10 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B61" s="99" t="str">
-        <x:v>IBIS</x:v>
+        <x:v>Focus Bracketing</x:v>
       </x:c>
       <x:c r="C61" s="99" t="str">
-        <x:v>sha256:f88432494f6ce6fd467acf866dcb7285209af0daa97f23211b4c2e9a2fca510a</x:v>
+        <x:v>sha256:faa653558ccc3ca42def02cffceb2449676221f3e2b701a95cb76c734a606a66</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -6764,20 +6766,9 @@
         <x:v>registration</x:v>
       </x:c>
       <x:c r="B62" s="99" t="str">
-        <x:v>Focus Bracketing</x:v>
+        <x:v>Lens IS switch</x:v>
       </x:c>
       <x:c r="C62" s="99" t="str">
-        <x:v>sha256:faa653558ccc3ca42def02cffceb2449676221f3e2b701a95cb76c734a606a66</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="99" t="str">
-        <x:v>registration</x:v>
-      </x:c>
-      <x:c r="B63" s="99" t="str">
-        <x:v>Lens IS switch</x:v>
-      </x:c>
-      <x:c r="C63" s="99" t="str">
         <x:v>sha256:77c1f08d541f8a95c354155213e1184f193765664d2faca4e6245806067b6735</x:v>
       </x:c>
     </x:row>

</xml_diff>